<commit_message>
Agregar Bogota Running y mapa del verano a palabras clave (Eventos Bogota)
</commit_message>
<xml_diff>
--- a/Palabras_Clave_Bogota.xlsx
+++ b/Palabras_Clave_Bogota.xlsx
@@ -7,7 +7,7 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Palabras clave" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -17,13 +17,16 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="1">
+  <fonts count="2">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <b val="1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -46,8 +49,9 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -413,16 +417,20 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B30"/>
+  <dimension ref="A1:B32"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="31" customWidth="1" min="1" max="1"/>
+    <col width="54" customWidth="1" min="2" max="2"/>
+  </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>categoria</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>palabra_clave</t>
         </is>
@@ -773,6 +781,30 @@
       <c r="B30" t="inlineStr">
         <is>
           <t>mapas Bogota</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>Eventos Bogota</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>Bogota Running</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>Eventos Bogota</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>mapa del verano</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Agregar Bogota running y Mapa festival del verano a Infraestructura
</commit_message>
<xml_diff>
--- a/Palabras_Clave_Bogota.xlsx
+++ b/Palabras_Clave_Bogota.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B32"/>
+  <dimension ref="A1:B34"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="31" customWidth="1" min="1" max="1"/>
@@ -808,6 +808,30 @@
         </is>
       </c>
     </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>Infraestructura</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>Bogota running</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>Infraestructura</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>Mapa festival del verano Bogota</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>